<commit_message>
Teaching assignment parser, PDF viewer, and department/offering updates
Add teaching assignment Excel parser, sample PDF documents, requirements doc, and refinements to upload preview, departments, course offerings, and OVPAA repository views.
</commit_message>
<xml_diff>
--- a/sample-uploads/sample_departments.xlsx
+++ b/sample-uploads/sample_departments.xlsx
@@ -397,7 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
+  <cols>
+    <col min="1" max="1" width="44.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,51 +417,84 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>College of Computer Studies</v>
+        <v>School of Social &amp; Natural Sciences</v>
       </c>
       <c r="B2" t="str">
-        <v>CCS</v>
+        <v>SSNS</v>
       </c>
       <c r="C2" t="str">
-        <v>Dr. Evelyn S. Marquez</v>
+        <v>Dr. Maria Elena Santos</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>College of Engineering</v>
+        <v>School of Business and Accountancy</v>
       </c>
       <c r="B3" t="str">
-        <v>COE</v>
+        <v>SBA</v>
       </c>
       <c r="C3" t="str">
-        <v>Engr. Ramon T. Villanueva</v>
+        <v>Dr. Teresita L. Gomez</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>College of Business and Accountancy</v>
+        <v>School of Computer &amp; Information Sciences</v>
       </c>
       <c r="B4" t="str">
-        <v>CBA</v>
+        <v>SCIS</v>
       </c>
       <c r="C4" t="str">
-        <v>Dr. Teresita L. Gomez</v>
+        <v>Dr. Evelyn S. Marquez</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>College of Arts and Sciences</v>
+        <v>College of Criminal Justice Education</v>
       </c>
       <c r="B5" t="str">
-        <v>CAS</v>
+        <v>CJE</v>
       </c>
       <c r="C5" t="str">
+        <v>Atty. Ramon D. Fernandez</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>School of Teacher Education</v>
+      </c>
+      <c r="B6" t="str">
+        <v>STE</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dr. Carmela V. Reyes</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>College of Engineering and Architecture</v>
+      </c>
+      <c r="B7" t="str">
+        <v>CEA</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Engr. Ramon T. Villanueva</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>School of Nursing &amp; Allied Health Sciences</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SNAHS</v>
+      </c>
+      <c r="C8" t="str">
         <v>Dr. Lourdes A. Bautista</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>